<commit_message>
Add investor list feature and admin/sales/booking improvements
- Add investor list pages (angel investors, VCs, family offices, incubators) with XLSX data source
- Add admin investor list product management pages
- Improve admin sales summary, bookings, and stats pages
- Update email templates and mailer
- Add sidebar navigation updates

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/angel-investor.xlsx
+++ b/data/angel-investor.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4e25a3dfa45fa3ed/Pitch to Priya/Investor List/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rkahu\priya-ahuja\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_F25DC773A252ABDACC1048A7C15A4C1A5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08A1E098-D2E8-444F-8139-6C8E535A9774}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{410B306D-91F7-42AD-B462-0382174F7D8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>